<commit_message>
refactor table equipment productivity
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Clone\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,12 +24,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Tên sản phẩm</t>
   </si>
   <si>
     <t>Tháng báo cáo</t>
+  </si>
+  <si>
+    <t>Ngày báo cáo</t>
   </si>
 </sst>
 </file>
@@ -66,7 +69,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFCFE2F3"/>
+        <fgColor theme="0"/>
         <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
@@ -116,16 +119,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -480,7 +483,8 @@
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
-    <col min="2" max="3" width="16.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.7109375" style="1" customWidth="1"/>
     <col min="4" max="9" width="12.5703125" style="1"/>
     <col min="10" max="10" width="15.7109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="15" style="1" customWidth="1"/>
@@ -495,35 +499,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
-      <c r="N1" s="5"/>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-      <c r="X1" s="3"/>
-      <c r="Y1" s="3"/>
-      <c r="Z1" s="3"/>
+      <c r="C1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
+      <c r="P1" s="3"/>
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+      <c r="S1" s="3"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+      <c r="X1" s="2"/>
+      <c r="Y1" s="2"/>
+      <c r="Z1" s="2"/>
     </row>
     <row r="2" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:26" ht="24" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
[Fix] common style to wrap text
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\KCVN\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Clone\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -494,11 +494,11 @@
     <col min="4" max="9" width="12.5703125" style="1"/>
     <col min="10" max="10" width="15.7109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="15" style="1" customWidth="1"/>
-    <col min="12" max="12" width="23.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="31.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="27" style="1" customWidth="1"/>
-    <col min="15" max="15" width="30.140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="21.85546875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="20" style="1" customWidth="1"/>
+    <col min="13" max="13" width="21.7109375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="20.42578125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="20.140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="17.42578125" style="1" customWidth="1"/>
     <col min="17" max="18" width="12.5703125" style="1"/>
     <col min="19" max="19" width="17.28515625" style="1" customWidth="1"/>
     <col min="20" max="16384" width="12.5703125" style="1"/>

</xml_diff>

<commit_message>
Revert "Merge branch 'hot-fix/common-style-sheet' into 'staging'"
This reverts merge request !965
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Clone\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\KCVN\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -494,11 +494,11 @@
     <col min="4" max="9" width="12.5703125" style="1"/>
     <col min="10" max="10" width="15.7109375" style="1" customWidth="1"/>
     <col min="11" max="11" width="15" style="1" customWidth="1"/>
-    <col min="12" max="12" width="20" style="1" customWidth="1"/>
-    <col min="13" max="13" width="21.7109375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="20.42578125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="20.140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="17.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23.5703125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="31.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="27" style="1" customWidth="1"/>
+    <col min="15" max="15" width="30.140625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="21.85546875" style="1" customWidth="1"/>
     <col min="17" max="18" width="12.5703125" style="1"/>
     <col min="19" max="19" width="17.28515625" style="1" customWidth="1"/>
     <col min="20" max="16384" width="12.5703125" style="1"/>

</xml_diff>

<commit_message>
[Fix] change column quantity report and change logic date completion rate
</commit_message>
<xml_diff>
--- a/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
+++ b/src/main/kotlin/com/kcvn/spm/assets/template/ExportQuantityReportTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\KCVN\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Clone\23-kcvn-spm-be\src\main\kotlin\com\kcvn\spm\assets\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -491,14 +491,15 @@
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
     <col min="2" max="2" width="16.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="31.7109375" style="1" customWidth="1"/>
-    <col min="4" max="9" width="12.5703125" style="1"/>
+    <col min="4" max="8" width="12.5703125" style="1"/>
+    <col min="9" max="9" width="14.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="15.7109375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="15" style="1" customWidth="1"/>
-    <col min="12" max="12" width="23.5703125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="31.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="27" style="1" customWidth="1"/>
-    <col min="15" max="15" width="30.140625" style="1" customWidth="1"/>
-    <col min="16" max="16" width="21.85546875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="18" style="1" customWidth="1"/>
+    <col min="13" max="13" width="22.28515625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="21.42578125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="19.28515625" style="1" customWidth="1"/>
+    <col min="16" max="16" width="20" style="1" customWidth="1"/>
     <col min="17" max="18" width="12.5703125" style="1"/>
     <col min="19" max="19" width="17.28515625" style="1" customWidth="1"/>
     <col min="20" max="16384" width="12.5703125" style="1"/>

</xml_diff>